<commit_message>
Add Parking Slots column to the Warehouse import template
Both copies (source templates/ and served frontend/public/templates/)
get a new "Parking Slots" column after Area sq ft, plus a matching
Legend & Rules explanation row.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/templates/Warehouse_Master_Import_Template.xlsx
+++ b/frontend/public/templates/Warehouse_Master_Import_Template.xlsx
@@ -399,31 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V10"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="17.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
-    <col min="12" max="12" width="14.83203125" customWidth="1"/>
-    <col min="13" max="13" width="15.83203125" customWidth="1"/>
-    <col min="14" max="14" width="14.83203125" customWidth="1"/>
-    <col min="15" max="15" width="15.83203125" customWidth="1"/>
-    <col min="16" max="16" width="14.83203125" customWidth="1"/>
-    <col min="17" max="17" width="14.83203125" customWidth="1"/>
-    <col min="18" max="18" width="20.83203125" customWidth="1"/>
-    <col min="19" max="19" width="14.83203125" customWidth="1"/>
-    <col min="20" max="20" width="14.83203125" customWidth="1"/>
-    <col min="21" max="21" width="14.83203125" customWidth="1"/>
-    <col min="22" max="22" width="15.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:W10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -457,39 +433,42 @@
         <v>Area sq ft</v>
       </c>
       <c r="K1" t="str">
+        <v>Parking Slots</v>
+      </c>
+      <c r="L1" t="str">
         <v>GSTIN</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Working Days</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Working Hours</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Contact Name</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Contact Phone</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Storage Type</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>Category</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>Pallet Positions *</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>Dim L (m)</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>Dim W (m)</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>Dim H (m)</v>
       </c>
-      <c r="V1" t="str">
+      <c r="W1" t="str">
         <v>Dispatch Flow</v>
       </c>
     </row>
@@ -524,40 +503,43 @@
       <c r="J2">
         <v>25000</v>
       </c>
-      <c r="K2" t="str">
+      <c r="K2">
+        <v>20</v>
+      </c>
+      <c r="L2" t="str">
         <v>33AAAAA0000A1Z5</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>Mon-Sat</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>09:00-19:00</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>Site Contact</v>
       </c>
-      <c r="O2" t="str">
+      <c r="P2" t="str">
         <v>9876500000</v>
       </c>
-      <c r="P2" t="str">
+      <c r="Q2" t="str">
         <v>SPR</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="R2" t="str">
         <v>Car Tyres</v>
       </c>
-      <c r="R2">
+      <c r="S2">
         <v>3000</v>
       </c>
-      <c r="S2">
+      <c r="T2">
         <v>1</v>
       </c>
-      <c r="T2">
+      <c r="U2">
         <v>1.5</v>
       </c>
-      <c r="U2">
+      <c r="V2">
         <v>1</v>
       </c>
-      <c r="V2" t="str">
+      <c r="W2" t="str">
         <v>Full Pallet</v>
       </c>
     </row>
@@ -608,24 +590,27 @@
         <v/>
       </c>
       <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
         <v>Drive-in</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="R3" t="str">
         <v>Truck Tyres-Radial</v>
       </c>
-      <c r="R3">
+      <c r="S3">
         <v>1200</v>
       </c>
-      <c r="S3">
+      <c r="T3">
         <v>1.5</v>
       </c>
-      <c r="T3">
+      <c r="U3">
         <v>1.8</v>
       </c>
-      <c r="U3">
+      <c r="V3">
         <v>1.2</v>
       </c>
-      <c r="V3" t="str">
+      <c r="W3" t="str">
         <v>Case Pick</v>
       </c>
     </row>
@@ -694,6 +679,9 @@
         <v/>
       </c>
       <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
         <v>Broken Case</v>
       </c>
     </row>
@@ -764,6 +752,9 @@
       <c r="V5" t="str">
         <v/>
       </c>
+      <c r="W5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -812,17 +803,17 @@
         <v/>
       </c>
       <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
         <v>Mix</v>
       </c>
-      <c r="Q6" t="str">
+      <c r="R6" t="str">
         <v>Uncategorized</v>
       </c>
-      <c r="R6">
+      <c r="S6">
         <v>5000</v>
       </c>
-      <c r="S6" t="str">
-        <v/>
-      </c>
       <c r="T6" t="str">
         <v/>
       </c>
@@ -830,6 +821,9 @@
         <v/>
       </c>
       <c r="V6" t="str">
+        <v/>
+      </c>
+      <c r="W6" t="str">
         <v>Full Pallet</v>
       </c>
     </row>
@@ -898,6 +892,9 @@
         <v/>
       </c>
       <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
         <v>Case Pick</v>
       </c>
     </row>
@@ -933,39 +930,42 @@
         <v>40000</v>
       </c>
       <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
         <v>33BBBBB1111B2Z6</v>
-      </c>
-      <c r="L8" t="str">
-        <v>24x7</v>
       </c>
       <c r="M8" t="str">
         <v>24x7</v>
       </c>
       <c r="N8" t="str">
+        <v>24x7</v>
+      </c>
+      <c r="O8" t="str">
         <v>Plant Manager</v>
       </c>
-      <c r="O8" t="str">
+      <c r="P8" t="str">
         <v>9876511111</v>
       </c>
-      <c r="P8" t="str">
+      <c r="Q8" t="str">
         <v>ASRS</v>
       </c>
-      <c r="Q8" t="str">
+      <c r="R8" t="str">
         <v>Water</v>
       </c>
-      <c r="R8">
+      <c r="S8">
         <v>8000</v>
       </c>
-      <c r="S8">
+      <c r="T8">
         <v>0.4</v>
       </c>
-      <c r="T8">
+      <c r="U8">
         <v>0.3</v>
       </c>
-      <c r="U8">
+      <c r="V8">
         <v>0.25</v>
       </c>
-      <c r="V8" t="str">
+      <c r="W8" t="str">
         <v>Full Pallet</v>
       </c>
     </row>
@@ -1016,17 +1016,17 @@
         <v/>
       </c>
       <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
         <v>Ground/Floor</v>
       </c>
-      <c r="Q9" t="str">
+      <c r="R9" t="str">
         <v>Carbonated</v>
       </c>
-      <c r="R9">
+      <c r="S9">
         <v>2000</v>
       </c>
-      <c r="S9" t="str">
-        <v/>
-      </c>
       <c r="T9" t="str">
         <v/>
       </c>
@@ -1034,6 +1034,9 @@
         <v/>
       </c>
       <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
         <v/>
       </c>
     </row>
@@ -1102,12 +1105,15 @@
         <v/>
       </c>
       <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
         <v>Full Pallet</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1115,9 +1121,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A13"/>
-  <cols>
-    <col min="1" max="1" width="100.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1193,12 +1196,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
-  <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
-    <col min="3" max="3" width="100.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:C21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1312,117 +1310,128 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>GSTIN</v>
+        <v>Parking Slots</v>
       </c>
       <c r="B11" t="str">
         <v>No</v>
       </c>
       <c r="C11" t="str">
-        <v>This facility's own GST registration number — distinct from any customer's GST number. No format enforced yet.</v>
+        <v>Whole number, 0 or more — how many vehicles can park in the yard at once. Generates that many numbered parking slots for this warehouse (Y1, Y2...). Leave blank/0 for a facility with no on-site parking — Yard Management simply does not apply to it.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Working Days</v>
+        <v>GSTIN</v>
       </c>
       <c r="B12" t="str">
         <v>No</v>
       </c>
       <c r="C12" t="str">
-        <v>Free text, e.g. "Mon-Sat" or "24x7".</v>
+        <v>This facility's own GST registration number — distinct from any customer's GST number. No format enforced yet.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Working Hours</v>
+        <v>Working Days</v>
       </c>
       <c r="B13" t="str">
         <v>No</v>
       </c>
       <c r="C13" t="str">
-        <v>Free text, e.g. "09:00-18:00" or "24x7".</v>
+        <v>Free text, e.g. "Mon-Sat" or "24x7".</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Contact Name</v>
+        <v>Working Hours</v>
       </c>
       <c r="B14" t="str">
         <v>No</v>
       </c>
       <c r="C14" t="str">
-        <v>Free text — the facility's primary point of contact.</v>
+        <v>Free text, e.g. "09:00-18:00" or "24x7".</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Contact Phone</v>
+        <v>Contact Name</v>
       </c>
       <c r="B15" t="str">
         <v>No</v>
       </c>
       <c r="C15" t="str">
-        <v>Free text.</v>
+        <v>Free text — the facility's primary point of contact.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Storage Type</v>
+        <v>Contact Phone</v>
       </c>
       <c r="B16" t="str">
         <v>No</v>
       </c>
       <c r="C16" t="str">
-        <v>One of: Ground/Floor, SPR, Drive-in, Mix, ASRS. Fill on a row to record one storage-type entry for this warehouse — use multiple rows (same Location Code) to break a warehouse down by storage type, each with its own Category, Pallet Positions, and dimensions. Don't combine "Mix" with specific storage-type rows for the same warehouse — pick one approach per warehouse.</v>
+        <v>Free text.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Category</v>
+        <v>Storage Type</v>
       </c>
       <c r="B17" t="str">
         <v>No</v>
       </c>
       <c r="C17" t="str">
-        <v>Must match a name in the Product Category master list (case-insensitive). Leave blank for "Uncategorized". This list is centrally managed — ask before typing a new category name, it will be rejected if not found. The same Category can appear against more than one Storage Type on the same warehouse (different Pallet count/dimensions each); what's not allowed is the same Storage Type + Category pair twice.</v>
+        <v>One of: Ground/Floor, SPR, Drive-in, Mix, ASRS. Fill on a row to record one storage-type entry for this warehouse — use multiple rows (same Location Code) to break a warehouse down by storage type, each with its own Category, Pallet Positions, and dimensions. Don't combine "Mix" with specific storage-type rows for the same warehouse — pick one approach per warehouse.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Pallet Positions *</v>
+        <v>Category</v>
       </c>
       <c r="B18" t="str">
-        <v>Only if Storage Type is filled on that row</v>
+        <v>No</v>
       </c>
       <c r="C18" t="str">
-        <v>Whole number, the pallet capacity for that specific Storage Type + Category combination (or the total, if using "Mix").</v>
+        <v>Must match a name in the Product Category master list (case-insensitive). Leave blank for "Uncategorized". This list is centrally managed — ask before typing a new category name, it will be rejected if not found. The same Category can appear against more than one Storage Type on the same warehouse (different Pallet count/dimensions each); what's not allowed is the same Storage Type + Category pair twice.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Dim L (m) / Dim W (m) / Dim H (m)</v>
+        <v>Pallet Positions *</v>
       </c>
       <c r="B19" t="str">
-        <v>No</v>
+        <v>Only if Storage Type is filled on that row</v>
       </c>
       <c r="C19" t="str">
-        <v>Positive numbers, in meters — the pallet-position dimensions for this Storage Type + Category combination. Optional; leave blank if not measured yet.</v>
+        <v>Whole number, the pallet capacity for that specific Storage Type + Category combination (or the total, if using "Mix").</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Dispatch Flow</v>
+        <v>Dim L (m) / Dim W (m) / Dim H (m)</v>
       </c>
       <c r="B20" t="str">
         <v>No</v>
       </c>
       <c r="C20" t="str">
+        <v>Positive numbers, in meters — the pallet-position dimensions for this Storage Type + Category combination. Optional; leave blank if not measured yet.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Dispatch Flow</v>
+      </c>
+      <c r="B21" t="str">
+        <v>No</v>
+      </c>
+      <c r="C21" t="str">
         <v>One of: Full Pallet, Case Pick, Broken Case. Fill on a row to record one dispatch capability for this warehouse — use multiple rows (same Location Code) to list more than one. A row can carry a Storage Type entry and a Dispatch Flow entry at the same time if convenient, or just one — they're independent, not linked to each other.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>